<commit_message>
Portal solo con la llave del carnet y zona por regularizar en el padrón
Portal del comerciante (como la pantalla P3 del Penpot):
- Se entra con DNI o código + llave del carnet, o con la llave sola al
  escanear el QR del reverso (nuevo botón, con el lector de Pagos).
- El PIN se quita del todo: sin ruta que lo genere, sin botón del
  personal y sin login que lo acepte. La migración 0017 borra pin_hash
  y los accesos que solo tenían PIN.

Importación del padrón:
- Un puesto sin zona o con una zona no registrada ya no cae en la
  primera zona sin avisar: queda en ella, paga con su tarifa y se marca
  "zona por regularizar" con lo que traía el libro (migración 0018).
- La zona se busca por nombre exacto; la búsqueda aproximada mandaba
  "Barrio Alto Salcedo" a la zona "SALCEDO".
- Sitios muestra la marca, un filtro y "Asignar zona…" (super_admin).

Pruebas: servidor 147/147, cliente 61/61, tsc y build de Vite.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos-prueba/padron-prueba-casos.xlsx
+++ b/datos-prueba/padron-prueba-casos.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="35">
   <si>
     <t>PADRÓN DE PRUEBA: CASOS ESPECIALES</t>
   </si>
@@ -92,6 +92,30 @@
   </si>
   <si>
     <t>Zona Norte</t>
+  </si>
+  <si>
+    <t>47120371</t>
+  </si>
+  <si>
+    <t>HILDA COAQUIRA RAMOS</t>
+  </si>
+  <si>
+    <t>CAS-D-005</t>
+  </si>
+  <si>
+    <t>Bloque D - Fila 3</t>
+  </si>
+  <si>
+    <t>47120372</t>
+  </si>
+  <si>
+    <t>EFRAIN TURPO CCAMA</t>
+  </si>
+  <si>
+    <t>CAS-D-006</t>
+  </si>
+  <si>
+    <t>Barrio Alto Salcedo</t>
   </si>
 </sst>
 </file>
@@ -490,7 +514,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -671,6 +695,70 @@
         <v>18</v>
       </c>
     </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I7">
+        <v>3</v>
+      </c>
+      <c r="J7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8">
+        <v>3</v>
+      </c>
+      <c r="J8" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>